<commit_message>
Interpolated CO Scores, Added Back Button, CO PO Targets Can be set Manually, Can Add CQI for all CO
</commit_message>
<xml_diff>
--- a/Test_data/New_Architecture/Complex_Scenario/Marks_Good.xlsx
+++ b/Test_data/New_Architecture/Complex_Scenario/Marks_Good.xlsx
@@ -463,7 +463,7 @@
         <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -473,10 +473,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -502,7 +502,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
         <v>4</v>
@@ -528,7 +528,7 @@
         <v>4</v>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -554,7 +554,7 @@
         <v>4</v>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -564,10 +564,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C12" t="n">
         <v>4</v>
@@ -593,7 +593,7 @@
         <v>4</v>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -603,10 +603,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C17" t="n">
         <v>4</v>
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
         <v>4</v>
@@ -668,10 +668,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -710,7 +710,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C24" t="n">
         <v>4</v>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C25" t="n">
         <v>4</v>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C26" t="n">
         <v>4</v>
@@ -772,7 +772,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C27" t="n">
         <v>4</v>
@@ -811,10 +811,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
         <v>4</v>
@@ -894,10 +894,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -910,7 +910,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -920,10 +920,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -936,7 +936,7 @@
         <v>4</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -962,7 +962,7 @@
         <v>3</v>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10" t="n">
         <v>4</v>
@@ -1001,7 +1001,7 @@
         <v>4</v>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13" t="n">
         <v>4</v>
@@ -1040,7 +1040,7 @@
         <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -1066,7 +1066,7 @@
         <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
@@ -1079,7 +1079,7 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
@@ -1089,10 +1089,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -1115,10 +1115,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22">
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22" t="n">
         <v>5</v>
@@ -1141,10 +1141,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
@@ -1157,7 +1157,7 @@
         <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C27" t="n">
         <v>4</v>
@@ -1248,7 +1248,7 @@
         <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1289,10 +1289,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -1302,10 +1302,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
         <v>4</v>
@@ -1354,10 +1354,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1383,7 +1383,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
         <v>4</v>
@@ -1409,7 +1409,7 @@
         <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1458,7 +1458,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
         <v>4</v>
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C16" t="n">
         <v>4</v>
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17" t="n">
         <v>4</v>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C18" t="n">
         <v>4</v>
@@ -1510,10 +1510,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -1523,10 +1523,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -1536,10 +1536,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -1552,7 +1552,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
@@ -1565,7 +1565,7 @@
         <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
@@ -1588,10 +1588,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
@@ -1601,7 +1601,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C26" t="n">
         <v>4</v>
@@ -1617,7 +1617,7 @@
         <v>4</v>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
@@ -1630,7 +1630,7 @@
         <v>5</v>
       </c>
       <c r="C28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
@@ -1640,10 +1640,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30">
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C30" t="n">
         <v>4</v>
@@ -1669,7 +1669,7 @@
         <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1710,10 +1710,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -1723,10 +1723,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1762,10 +1762,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -1788,10 +1788,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -1804,7 +1804,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -1814,7 +1814,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C10" t="n">
         <v>4</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C11" t="n">
         <v>4</v>
@@ -1840,10 +1840,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1869,7 +1869,7 @@
         <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -1921,7 +1921,7 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
@@ -1947,7 +1947,7 @@
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
         <v>4</v>
@@ -1973,7 +1973,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
@@ -1983,7 +1983,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C23" t="n">
         <v>4</v>
@@ -2025,7 +2025,7 @@
         <v>4</v>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C27" t="n">
         <v>3</v>
@@ -2048,10 +2048,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -2061,10 +2061,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C31" t="n">
         <v>4</v>
@@ -2144,7 +2144,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
         <v>4</v>
@@ -2160,7 +2160,7 @@
         <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -2170,10 +2170,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -2183,7 +2183,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6" t="n">
         <v>4</v>
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C8" t="n">
         <v>4</v>
@@ -2222,10 +2222,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -2235,7 +2235,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10" t="n">
         <v>4</v>
@@ -2248,10 +2248,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -2274,7 +2274,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C13" t="n">
         <v>4</v>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C14" t="n">
         <v>4</v>
@@ -2303,7 +2303,7 @@
         <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -2326,10 +2326,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
@@ -2339,10 +2339,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
@@ -2352,10 +2352,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -2368,7 +2368,7 @@
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -2394,7 +2394,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
@@ -2417,10 +2417,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
@@ -2430,10 +2430,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
@@ -2446,7 +2446,7 @@
         <v>4</v>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
@@ -2456,7 +2456,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C27" t="n">
         <v>4</v>
@@ -2469,10 +2469,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -2482,10 +2482,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -2498,7 +2498,7 @@
         <v>4</v>
       </c>
       <c r="C30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31">
@@ -2511,7 +2511,7 @@
         <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2555,7 +2555,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -2568,7 +2568,7 @@
         <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -2581,7 +2581,7 @@
         <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -2607,7 +2607,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
         <v>4</v>
@@ -2630,7 +2630,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
         <v>4</v>
@@ -2643,10 +2643,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -2659,7 +2659,7 @@
         <v>4</v>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -2669,7 +2669,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C11" t="n">
         <v>4</v>
@@ -2695,7 +2695,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C13" t="n">
         <v>4</v>
@@ -2721,7 +2721,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C15" t="n">
         <v>4</v>
@@ -2734,10 +2734,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17" t="n">
         <v>4</v>
@@ -2763,7 +2763,7 @@
         <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
@@ -2773,10 +2773,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -2799,10 +2799,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -2812,10 +2812,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
@@ -2838,10 +2838,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25">
@@ -2851,10 +2851,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
@@ -2864,10 +2864,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27">
@@ -2880,7 +2880,7 @@
         <v>4</v>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
@@ -2903,10 +2903,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
@@ -2916,7 +2916,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C30" t="n">
         <v>4</v>
@@ -2993,22 +2993,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E2" t="n">
         <v>9</v>
       </c>
       <c r="F2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -3021,19 +3021,19 @@
         <v>9</v>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
         <v>8</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F3" t="n">
         <v>7</v>
       </c>
       <c r="G3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -3043,22 +3043,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" t="n">
         <v>7</v>
       </c>
       <c r="D4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -3068,22 +3068,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D5" t="n">
         <v>9</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F5" t="n">
         <v>9</v>
       </c>
       <c r="G5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -3096,19 +3096,19 @@
         <v>7</v>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D6" t="n">
         <v>9</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -3121,19 +3121,19 @@
         <v>9</v>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G7" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -3143,22 +3143,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D8" t="n">
         <v>8</v>
       </c>
       <c r="E8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -3171,19 +3171,19 @@
         <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F9" t="n">
         <v>7</v>
       </c>
       <c r="G9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -3193,19 +3193,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D10" t="n">
         <v>8</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G10" t="n">
         <v>8</v>
@@ -3221,19 +3221,19 @@
         <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D11" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G11" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -3246,19 +3246,19 @@
         <v>7</v>
       </c>
       <c r="C12" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D12" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E12" t="n">
         <v>9</v>
       </c>
       <c r="F12" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -3271,16 +3271,16 @@
         <v>9</v>
       </c>
       <c r="C13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G13" t="n">
         <v>7</v>
@@ -3296,19 +3296,19 @@
         <v>9</v>
       </c>
       <c r="C14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D14" t="n">
         <v>9</v>
       </c>
       <c r="E14" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G14" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -3318,22 +3318,22 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C15" t="n">
         <v>7</v>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -3343,22 +3343,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C16" t="n">
         <v>7</v>
       </c>
       <c r="D16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F16" t="n">
         <v>7</v>
       </c>
       <c r="G16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
@@ -3368,22 +3368,22 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C17" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E17" t="n">
         <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18">
@@ -3393,19 +3393,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D18" t="n">
         <v>9</v>
       </c>
       <c r="E18" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G18" t="n">
         <v>8</v>
@@ -3430,10 +3430,10 @@
         <v>8</v>
       </c>
       <c r="F19" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20">
@@ -3443,10 +3443,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D20" t="n">
         <v>8</v>
@@ -3455,10 +3455,10 @@
         <v>8</v>
       </c>
       <c r="F20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21">
@@ -3468,22 +3468,22 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C21" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D21" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
         <v>7</v>
       </c>
       <c r="F21" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G21" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22">
@@ -3493,22 +3493,22 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C22" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D22" t="n">
         <v>8</v>
       </c>
       <c r="E22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F22" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G22" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
@@ -3524,13 +3524,13 @@
         <v>7</v>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E23" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G23" t="n">
         <v>7</v>
@@ -3543,13 +3543,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D24" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
         <v>8</v>
@@ -3568,22 +3568,22 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C25" t="n">
         <v>8</v>
       </c>
       <c r="D25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26">
@@ -3593,19 +3593,19 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C26" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D26" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E26" t="n">
         <v>7</v>
       </c>
       <c r="F26" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G26" t="n">
         <v>7</v>
@@ -3618,7 +3618,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C27" t="n">
         <v>7</v>
@@ -3630,7 +3630,7 @@
         <v>8</v>
       </c>
       <c r="F27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G27" t="n">
         <v>9</v>
@@ -3643,22 +3643,22 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D28" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E28" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F28" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G28" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29">
@@ -3668,19 +3668,19 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C29" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D29" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F29" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G29" t="n">
         <v>8</v>
@@ -3693,22 +3693,22 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C30" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D30" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E30" t="n">
         <v>8</v>
       </c>
       <c r="F30" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G30" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31">
@@ -3721,19 +3721,19 @@
         <v>7</v>
       </c>
       <c r="C31" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D31" t="n">
         <v>8</v>
       </c>
       <c r="E31" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F31" t="n">
         <v>8</v>
       </c>
       <c r="G31" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -3794,7 +3794,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
         <v>2</v>
@@ -3819,10 +3819,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
@@ -3831,7 +3831,7 @@
         <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3" t="n">
         <v>2</v>
@@ -3847,7 +3847,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
         <v>2</v>
@@ -3875,16 +3875,16 @@
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
         <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -3897,7 +3897,7 @@
         <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
         <v>3</v>
@@ -3909,7 +3909,7 @@
         <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -3919,22 +3919,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>2</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -3947,19 +3947,19 @@
         <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -3969,13 +3969,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
         <v>2</v>
@@ -3984,7 +3984,7 @@
         <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -3994,13 +3994,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
         <v>2</v>
@@ -4019,13 +4019,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C11" t="n">
         <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
         <v>2</v>
@@ -4044,13 +4044,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
         <v>2</v>
@@ -4059,7 +4059,7 @@
         <v>2</v>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -4069,13 +4069,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
         <v>3</v>
@@ -4094,7 +4094,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C14" t="n">
         <v>2</v>
@@ -4109,7 +4109,7 @@
         <v>2</v>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -4119,7 +4119,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n">
         <v>2</v>
@@ -4128,13 +4128,13 @@
         <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
         <v>2</v>
       </c>
       <c r="G15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -4144,22 +4144,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" t="n">
         <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -4178,10 +4178,10 @@
         <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G17" t="n">
         <v>3</v>
@@ -4203,7 +4203,7 @@
         <v>2</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
         <v>2</v>
@@ -4225,13 +4225,13 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
@@ -4244,16 +4244,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
         <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
         <v>2</v>
@@ -4294,22 +4294,22 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -4322,7 +4322,7 @@
         <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
         <v>3</v>
@@ -4334,7 +4334,7 @@
         <v>3</v>
       </c>
       <c r="G23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -4347,16 +4347,16 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G24" t="n">
         <v>2</v>
@@ -4369,7 +4369,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C25" t="n">
         <v>3</v>
@@ -4378,13 +4378,13 @@
         <v>2</v>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -4394,22 +4394,22 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C26" t="n">
         <v>3</v>
       </c>
       <c r="D26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -4419,16 +4419,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D27" t="n">
         <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F27" t="n">
         <v>3</v>
@@ -4447,7 +4447,7 @@
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D28" t="n">
         <v>2</v>
@@ -4478,13 +4478,13 @@
         <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -4497,13 +4497,13 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D30" t="n">
         <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F30" t="n">
         <v>3</v>
@@ -4519,10 +4519,10 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
         <v>2</v>
@@ -4531,10 +4531,10 @@
         <v>2</v>
       </c>
       <c r="F31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>